<commit_message>
- revise field_patterns.yaml, version
</commit_message>
<xml_diff>
--- a/data/12.09鋐利-中磊( 进口）-蜂鸣器.xlsx
+++ b/data/12.09鋐利-中磊( 进口）-蜂鸣器.xlsx
@@ -1,21 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.87\custom\1.进出货报关资料(IDEAL）\苏州众诚国际-中磊\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Liou\Projects\AutoConvert_v3.8.0\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3414A305-182F-486E-AFAB-C145B0C3DBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8205" activeTab="1"/>
+    <workbookView xWindow="40224" yWindow="1860" windowWidth="23040" windowHeight="11808" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INVOICE" sheetId="1" r:id="rId1"/>
     <sheet name="PACKING" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -519,18 +533,18 @@
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">2250303826/1.1 </t>
-    <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
     <t>PQDHL018-USD2025120900001</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">2250303826.1.1 </t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
     <numFmt numFmtId="176" formatCode="0.00_ "/>
     <numFmt numFmtId="177" formatCode="yyyy/m/d;@"/>
@@ -544,7 +558,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -603,7 +617,7 @@
     <font>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -622,7 +636,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -647,7 +661,7 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -656,7 +670,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -665,7 +679,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -686,7 +700,7 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -719,7 +733,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="新細明體"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -919,422 +933,405 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="1" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="176" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="180" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规_Sheet1_1" xfId="3"/>
-    <cellStyle name="一般_OMRON" xfId="2"/>
-    <cellStyle name="一般_OMRON海運出口" xfId="1"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="一般_OMRON" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="一般_OMRON海運出口" xfId="1" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="常规_Sheet1_1" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1371,7 +1368,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 1" descr="TT{_GCLFJ`S{T0HZ~J%_V[2"/>
+        <xdr:cNvPr id="3" name="Picture 1" descr="TT{_GCLFJ`S{T0HZ~J%_V[2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1454,7 +1457,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="TT{_GCLFJ`S{T0HZ~J%_V[2"/>
+        <xdr:cNvPr id="2" name="Picture 1" descr="TT{_GCLFJ`S{T0HZ~J%_V[2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -1777,81 +1786,81 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O28"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="22.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="24.6"/>
   <cols>
-    <col min="1" max="1" width="6.125" style="81" customWidth="1"/>
-    <col min="2" max="2" width="11.375" style="81" customWidth="1"/>
-    <col min="3" max="3" width="14.25" style="81" customWidth="1"/>
-    <col min="4" max="4" width="9" style="81"/>
-    <col min="5" max="5" width="10.125" style="81" customWidth="1"/>
-    <col min="6" max="6" width="6.875" style="81" customWidth="1"/>
-    <col min="7" max="9" width="9" style="81"/>
-    <col min="10" max="10" width="5.875" style="81" customWidth="1"/>
-    <col min="11" max="11" width="5.5" style="81" customWidth="1"/>
-    <col min="12" max="12" width="7.125" style="81" customWidth="1"/>
-    <col min="13" max="13" width="7" style="81" customWidth="1"/>
-    <col min="14" max="14" width="7.125" style="81" customWidth="1"/>
-    <col min="15" max="15" width="7.875" style="81" customWidth="1"/>
-    <col min="16" max="16384" width="9" style="81"/>
+    <col min="1" max="1" width="6.125" style="76" customWidth="1"/>
+    <col min="2" max="2" width="11.375" style="76" customWidth="1"/>
+    <col min="3" max="3" width="14.25" style="76" customWidth="1"/>
+    <col min="4" max="4" width="17.25" style="76" customWidth="1"/>
+    <col min="5" max="5" width="10.125" style="76" customWidth="1"/>
+    <col min="6" max="6" width="6.875" style="76" customWidth="1"/>
+    <col min="7" max="9" width="9" style="76"/>
+    <col min="10" max="10" width="5.875" style="76" customWidth="1"/>
+    <col min="11" max="11" width="5.5" style="76" customWidth="1"/>
+    <col min="12" max="12" width="7.125" style="76" customWidth="1"/>
+    <col min="13" max="13" width="7" style="76" customWidth="1"/>
+    <col min="14" max="14" width="7.125" style="76" customWidth="1"/>
+    <col min="15" max="15" width="7.875" style="76" customWidth="1"/>
+    <col min="16" max="16384" width="9" style="76"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="23.25">
-      <c r="A1" s="142" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="143"/>
-      <c r="J1" s="143"/>
-      <c r="K1" s="143"/>
-      <c r="L1" s="143"/>
-      <c r="M1" s="143"/>
-      <c r="N1" s="143"/>
-      <c r="O1" s="144"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
+      <c r="I1" s="134"/>
+      <c r="J1" s="134"/>
+      <c r="K1" s="134"/>
+      <c r="L1" s="134"/>
+      <c r="M1" s="134"/>
+      <c r="N1" s="134"/>
+      <c r="O1" s="135"/>
     </row>
     <row r="2" spans="1:15">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="82" t="s">
+      <c r="B2" s="78"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
       <c r="O2" s="11"/>
     </row>
     <row r="3" spans="1:15" ht="17.25" customHeight="1">
-      <c r="A3" s="127" t="s">
+      <c r="A3" s="119" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="38" t="s">
+      <c r="B3" s="33"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="84"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="84"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="46"/>
       <c r="J3" s="17"/>
       <c r="K3" s="17"/>
       <c r="L3" s="17"/>
@@ -1860,19 +1869,19 @@
       <c r="O3" s="11"/>
     </row>
     <row r="4" spans="1:15">
-      <c r="A4" s="139" t="s">
+      <c r="A4" s="130" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="140"/>
-      <c r="C4" s="140"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="87" t="s">
+      <c r="B4" s="131"/>
+      <c r="C4" s="131"/>
+      <c r="D4" s="132"/>
+      <c r="E4" s="81" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="88"/>
-      <c r="G4" s="88"/>
+      <c r="F4" s="82"/>
+      <c r="G4" s="82"/>
       <c r="H4" s="12"/>
-      <c r="I4" s="84"/>
+      <c r="I4" s="46"/>
       <c r="J4" s="17"/>
       <c r="K4" s="17"/>
       <c r="L4" s="17"/>
@@ -1881,15 +1890,15 @@
       <c r="O4" s="11"/>
     </row>
     <row r="5" spans="1:15">
-      <c r="A5" s="139"/>
-      <c r="B5" s="140"/>
-      <c r="C5" s="140"/>
-      <c r="D5" s="141"/>
-      <c r="E5" s="89"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="84"/>
-      <c r="H5" s="84"/>
-      <c r="I5" s="84"/>
+      <c r="A5" s="130"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="132"/>
+      <c r="E5" s="83"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
+      <c r="I5" s="46"/>
       <c r="J5" s="17"/>
       <c r="K5" s="17"/>
       <c r="L5" s="17"/>
@@ -1898,15 +1907,15 @@
       <c r="O5" s="11"/>
     </row>
     <row r="6" spans="1:15">
-      <c r="A6" s="39"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="91"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
+      <c r="A6" s="37"/>
+      <c r="B6" s="84"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
       <c r="J6" s="18"/>
       <c r="K6" s="18"/>
       <c r="L6" s="18"/>
@@ -1915,19 +1924,19 @@
       <c r="O6" s="19"/>
     </row>
     <row r="7" spans="1:15">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="93"/>
-      <c r="C7" s="94"/>
-      <c r="D7" s="95"/>
-      <c r="E7" s="44" t="s">
+      <c r="B7" s="87"/>
+      <c r="C7" s="88"/>
+      <c r="D7" s="89"/>
+      <c r="E7" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="94"/>
-      <c r="G7" s="94"/>
-      <c r="H7" s="94"/>
-      <c r="I7" s="94"/>
+      <c r="F7" s="88"/>
+      <c r="G7" s="88"/>
+      <c r="H7" s="88"/>
+      <c r="I7" s="88"/>
       <c r="J7" s="20"/>
       <c r="K7" s="21"/>
       <c r="L7" s="21"/>
@@ -1936,17 +1945,17 @@
       <c r="O7" s="22"/>
     </row>
     <row r="8" spans="1:15">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="35"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="9"/>
-      <c r="D8" s="96"/>
-      <c r="E8" s="89"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-      <c r="H8" s="84"/>
-      <c r="I8" s="84"/>
+      <c r="D8" s="90"/>
+      <c r="E8" s="83"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
       <c r="J8" s="21"/>
       <c r="K8" s="21"/>
       <c r="L8" s="21"/>
@@ -1955,17 +1964,17 @@
       <c r="O8" s="22"/>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="139" t="s">
+      <c r="A9" s="130" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="140"/>
-      <c r="C9" s="140"/>
-      <c r="D9" s="141"/>
-      <c r="E9" s="145"/>
-      <c r="F9" s="146"/>
-      <c r="G9" s="146"/>
-      <c r="H9" s="146"/>
-      <c r="I9" s="146"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="136"/>
+      <c r="F9" s="137"/>
+      <c r="G9" s="137"/>
+      <c r="H9" s="137"/>
+      <c r="I9" s="137"/>
       <c r="J9" s="23"/>
       <c r="K9" s="23"/>
       <c r="L9" s="23"/>
@@ -1974,15 +1983,15 @@
       <c r="O9" s="24"/>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="139"/>
-      <c r="B10" s="140"/>
-      <c r="C10" s="140"/>
-      <c r="D10" s="141"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="84"/>
-      <c r="G10" s="84"/>
-      <c r="H10" s="84"/>
-      <c r="I10" s="84"/>
+      <c r="A10" s="130"/>
+      <c r="B10" s="131"/>
+      <c r="C10" s="131"/>
+      <c r="D10" s="132"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
       <c r="J10" s="23"/>
       <c r="K10" s="23"/>
       <c r="L10" s="23"/>
@@ -1991,80 +2000,80 @@
       <c r="O10" s="24"/>
     </row>
     <row r="11" spans="1:15">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="94"/>
-      <c r="C11" s="94"/>
-      <c r="D11" s="95"/>
-      <c r="E11" s="44" t="s">
+      <c r="B11" s="88"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="89"/>
+      <c r="E11" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="94"/>
-      <c r="G11" s="94"/>
-      <c r="H11" s="94"/>
-      <c r="I11" s="94"/>
-      <c r="J11" s="94"/>
-      <c r="K11" s="94"/>
-      <c r="L11" s="94"/>
-      <c r="M11" s="94"/>
-      <c r="N11" s="94"/>
-      <c r="O11" s="95"/>
+      <c r="F11" s="88"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
+      <c r="K11" s="88"/>
+      <c r="L11" s="88"/>
+      <c r="M11" s="88"/>
+      <c r="N11" s="88"/>
+      <c r="O11" s="89"/>
     </row>
     <row r="12" spans="1:15" ht="20.25" customHeight="1">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="85"/>
-      <c r="E12" s="38" t="s">
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="79"/>
+      <c r="E12" s="36" t="s">
         <v>43</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="25"/>
-      <c r="N12" s="25"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+      <c r="N12" s="17"/>
       <c r="O12" s="11"/>
     </row>
     <row r="13" spans="1:15">
-      <c r="A13" s="41"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="91"/>
-      <c r="E13" s="92"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="97"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
+      <c r="A13" s="39"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="85"/>
+      <c r="E13" s="86"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="91"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
       <c r="O13" s="19"/>
     </row>
     <row r="14" spans="1:15">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="94"/>
-      <c r="C14" s="44" t="s">
+      <c r="B14" s="88"/>
+      <c r="C14" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="95"/>
-      <c r="E14" s="83" t="s">
+      <c r="D14" s="89"/>
+      <c r="E14" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="49"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="46"/>
       <c r="J14" s="16"/>
       <c r="K14" s="16"/>
       <c r="L14" s="16"/>
@@ -2073,255 +2082,255 @@
       <c r="O14" s="11"/>
     </row>
     <row r="15" spans="1:15">
-      <c r="A15" s="147"/>
-      <c r="B15" s="148"/>
-      <c r="C15" s="147"/>
-      <c r="D15" s="148"/>
-      <c r="E15" s="98"/>
-      <c r="F15" s="84"/>
-      <c r="G15" s="84"/>
-      <c r="H15" s="84"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="25"/>
-      <c r="N15" s="25"/>
+      <c r="A15" s="138"/>
+      <c r="B15" s="139"/>
+      <c r="C15" s="138"/>
+      <c r="D15" s="139"/>
+      <c r="E15" s="92"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
       <c r="O15" s="11"/>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="1"/>
       <c r="B16" s="2"/>
       <c r="C16" s="13"/>
-      <c r="D16" s="99"/>
-      <c r="E16" s="98"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="92"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="84"/>
-      <c r="H16" s="84"/>
-      <c r="I16" s="49"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="25"/>
-      <c r="N16" s="25"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="17"/>
+      <c r="N16" s="17"/>
       <c r="O16" s="11"/>
     </row>
     <row r="17" spans="1:15">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="95"/>
-      <c r="C17" s="82" t="s">
+      <c r="B17" s="89"/>
+      <c r="C17" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="58"/>
-      <c r="E17" s="98"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="92"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="N17" s="25"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
       <c r="O17" s="11"/>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="6"/>
       <c r="B18" s="14"/>
-      <c r="C18" s="149"/>
-      <c r="D18" s="150"/>
-      <c r="E18" s="100" t="s">
+      <c r="C18" s="140"/>
+      <c r="D18" s="141"/>
+      <c r="E18" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="F18" s="40" t="s">
+      <c r="F18" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="25"/>
-      <c r="M18" s="25"/>
-      <c r="N18" s="25"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="17"/>
       <c r="O18" s="11"/>
     </row>
-    <row r="19" spans="1:15" ht="24">
-      <c r="A19" s="120" t="s">
+    <row r="19" spans="1:15" ht="36">
+      <c r="A19" s="112" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="121" t="s">
+      <c r="B19" s="113" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="121" t="s">
+      <c r="C19" s="113" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="122" t="s">
+      <c r="D19" s="114" t="s">
         <v>16</v>
       </c>
-      <c r="E19" s="121" t="s">
+      <c r="E19" s="113" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="121" t="s">
+      <c r="F19" s="113" t="s">
         <v>18</v>
       </c>
-      <c r="G19" s="121" t="s">
+      <c r="G19" s="113" t="s">
         <v>19</v>
       </c>
-      <c r="H19" s="121" t="s">
+      <c r="H19" s="113" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="121" t="s">
+      <c r="I19" s="113" t="s">
         <v>21</v>
       </c>
-      <c r="J19" s="123" t="s">
+      <c r="J19" s="115" t="s">
         <v>22</v>
       </c>
-      <c r="K19" s="123" t="s">
+      <c r="K19" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="L19" s="124" t="s">
+      <c r="L19" s="116" t="s">
         <v>24</v>
       </c>
-      <c r="M19" s="125" t="s">
+      <c r="M19" s="117" t="s">
         <v>25</v>
       </c>
-      <c r="N19" s="124" t="s">
+      <c r="N19" s="116" t="s">
         <v>26</v>
       </c>
-      <c r="O19" s="126" t="s">
+      <c r="O19" s="118" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:15" s="79" customFormat="1" ht="20.25" customHeight="1">
-      <c r="A20" s="28" t="s">
+    <row r="20" spans="1:15" s="74" customFormat="1" ht="20.25" customHeight="1">
+      <c r="A20" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="75" t="s">
+      <c r="B20" s="70" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="75" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" s="29" t="s">
+      <c r="C20" s="70" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="75">
+      <c r="E20" s="70">
         <v>5000</v>
       </c>
-      <c r="F20" s="101" t="s">
+      <c r="F20" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="G20" s="102">
+      <c r="G20" s="95">
         <v>0.5</v>
       </c>
-      <c r="H20" s="103" t="s">
+      <c r="H20" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="I20" s="78">
+      <c r="I20" s="73">
         <f t="shared" ref="I20" si="0">ROUND(E20*G20,2)</f>
         <v>2500</v>
       </c>
-      <c r="J20" s="75" t="s">
+      <c r="J20" s="70" t="s">
         <v>45</v>
       </c>
-      <c r="K20" s="75"/>
-      <c r="L20" s="29" t="s">
+      <c r="K20" s="70"/>
+      <c r="L20" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="M20" s="29" t="s">
+      <c r="M20" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="N20" s="29" t="s">
+      <c r="N20" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="O20" s="130">
+      <c r="O20" s="121">
         <f>PACKING!H22</f>
         <v>2.5</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="16.5" customHeight="1">
-      <c r="A21" s="104"/>
-      <c r="J21" s="105"/>
-      <c r="K21" s="105"/>
-      <c r="L21" s="105"/>
-      <c r="M21" s="105"/>
-      <c r="N21" s="105"/>
-      <c r="O21" s="106"/>
+      <c r="A21" s="96"/>
+      <c r="J21" s="97"/>
+      <c r="K21" s="97"/>
+      <c r="L21" s="97"/>
+      <c r="M21" s="97"/>
+      <c r="N21" s="97"/>
+      <c r="O21" s="98"/>
     </row>
     <row r="22" spans="1:15">
-      <c r="A22" s="107"/>
-      <c r="B22" s="108"/>
-      <c r="C22" s="138" t="s">
+      <c r="A22" s="99"/>
+      <c r="B22" s="100"/>
+      <c r="C22" s="129" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="138"/>
-      <c r="E22" s="109">
+      <c r="D22" s="129"/>
+      <c r="E22" s="101">
         <f>SUM(E20:E21)</f>
         <v>5000</v>
       </c>
       <c r="F22" s="15"/>
-      <c r="G22" s="110"/>
-      <c r="H22" s="110"/>
-      <c r="I22" s="111">
+      <c r="G22" s="102"/>
+      <c r="H22" s="102"/>
+      <c r="I22" s="103">
         <f>SUM(I20:I21)</f>
         <v>2500</v>
       </c>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-      <c r="O22" s="111">
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
+      <c r="L22" s="26"/>
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="103">
         <f>SUM(O20:O21)</f>
         <v>2.5</v>
       </c>
     </row>
     <row r="24" spans="1:15">
-      <c r="B24" s="132" t="s">
+      <c r="B24" s="123" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="132" t="s">
+      <c r="C24" s="123" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="79"/>
+      <c r="D24" s="74"/>
     </row>
     <row r="25" spans="1:15">
-      <c r="B25" s="132" t="s">
+      <c r="B25" s="123" t="s">
         <v>68</v>
       </c>
-      <c r="C25" s="133">
+      <c r="C25" s="124">
         <v>2358</v>
       </c>
-      <c r="D25" s="79"/>
+      <c r="D25" s="74"/>
     </row>
     <row r="26" spans="1:15">
-      <c r="B26" s="132" t="s">
+      <c r="B26" s="123" t="s">
         <v>69</v>
       </c>
-      <c r="C26" s="132" t="s">
+      <c r="C26" s="123" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="79"/>
+      <c r="D26" s="74"/>
     </row>
     <row r="27" spans="1:15">
-      <c r="B27" s="132" t="s">
+      <c r="B27" s="123" t="s">
         <v>71</v>
       </c>
-      <c r="C27" s="132" t="s">
+      <c r="C27" s="123" t="s">
         <v>72</v>
       </c>
-      <c r="D27" s="79"/>
+      <c r="D27" s="74"/>
     </row>
     <row r="28" spans="1:15">
-      <c r="F28" s="112" t="s">
+      <c r="F28" s="104" t="s">
         <v>62</v>
       </c>
-      <c r="G28" s="113"/>
-      <c r="H28" s="113"/>
-      <c r="I28" s="113"/>
+      <c r="G28" s="105"/>
+      <c r="H28" s="105"/>
+      <c r="I28" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2342,466 +2351,466 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.5" style="30" customWidth="1"/>
-    <col min="2" max="2" width="15.125" style="30" customWidth="1"/>
-    <col min="3" max="3" width="12.375" style="30" customWidth="1"/>
-    <col min="4" max="4" width="9" style="30"/>
-    <col min="5" max="5" width="5.25" style="30" customWidth="1"/>
-    <col min="6" max="6" width="10.125" style="30"/>
-    <col min="7" max="7" width="5.375" style="30" customWidth="1"/>
-    <col min="8" max="8" width="7" style="30" customWidth="1"/>
-    <col min="9" max="9" width="8.375" style="30" customWidth="1"/>
-    <col min="10" max="10" width="12.875" style="30" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="30"/>
+    <col min="1" max="1" width="5.5" customWidth="1"/>
+    <col min="2" max="2" width="15.125" customWidth="1"/>
+    <col min="3" max="3" width="12.375" customWidth="1"/>
+    <col min="5" max="5" width="5.25" customWidth="1"/>
+    <col min="6" max="6" width="10.125"/>
+    <col min="7" max="7" width="5.375" customWidth="1"/>
+    <col min="8" max="8" width="7" customWidth="1"/>
+    <col min="9" max="9" width="8.375" customWidth="1"/>
+    <col min="10" max="10" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20.25">
-      <c r="A1" s="161" t="s">
+    <row r="1" spans="1:10" ht="21">
+      <c r="A1" s="146" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="162"/>
-      <c r="C1" s="162"/>
-      <c r="D1" s="162"/>
-      <c r="E1" s="162"/>
-      <c r="F1" s="162"/>
-      <c r="G1" s="162"/>
-      <c r="H1" s="162"/>
-      <c r="I1" s="162"/>
-      <c r="J1" s="163"/>
-    </row>
-    <row r="2" spans="1:10" ht="14.25">
-      <c r="A2" s="80" t="s">
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="148"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="75" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="56"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="56" t="s">
+      <c r="B2" s="45"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
       <c r="J2" s="11"/>
     </row>
-    <row r="3" spans="1:10" ht="15">
-      <c r="A3" s="128" t="s">
+    <row r="3" spans="1:10">
+      <c r="A3" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="38" t="str">
+      <c r="B3" s="33"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="36" t="str">
         <f>INVOICE!E3</f>
         <v>VF-1141209-01</v>
       </c>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
       <c r="J3" s="11"/>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A4" s="165" t="s">
+      <c r="A4" s="153" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="166"/>
-      <c r="C4" s="166"/>
-      <c r="D4" s="166"/>
-      <c r="E4" s="167"/>
-      <c r="F4" s="38" t="str">
+      <c r="B4" s="154"/>
+      <c r="C4" s="154"/>
+      <c r="D4" s="154"/>
+      <c r="E4" s="155"/>
+      <c r="F4" s="36" t="str">
         <f>INVOICE!E4</f>
         <v>2025.12.09</v>
       </c>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
       <c r="J4" s="11"/>
     </row>
-    <row r="5" spans="1:10" ht="14.25">
-      <c r="A5" s="165"/>
-      <c r="B5" s="166"/>
-      <c r="C5" s="166"/>
-      <c r="D5" s="166"/>
-      <c r="E5" s="167"/>
-      <c r="F5" s="134" t="s">
+    <row r="5" spans="1:10">
+      <c r="A5" s="153"/>
+      <c r="B5" s="154"/>
+      <c r="C5" s="154"/>
+      <c r="D5" s="154"/>
+      <c r="E5" s="155"/>
+      <c r="F5" s="125" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="135"/>
-      <c r="H5" s="135"/>
-      <c r="I5" s="135"/>
+      <c r="G5" s="126"/>
+      <c r="H5" s="126"/>
+      <c r="I5" s="126"/>
       <c r="J5" s="11"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="168"/>
-      <c r="B6" s="169"/>
-      <c r="C6" s="169"/>
-      <c r="D6" s="169"/>
-      <c r="E6" s="170"/>
-      <c r="F6" s="136" t="s">
-        <v>78</v>
-      </c>
-      <c r="G6" s="137"/>
-      <c r="H6" s="137"/>
-      <c r="I6" s="137"/>
-      <c r="J6" s="43"/>
-    </row>
-    <row r="7" spans="1:10" ht="14.25">
-      <c r="A7" s="44" t="s">
+      <c r="A6" s="156"/>
+      <c r="B6" s="157"/>
+      <c r="C6" s="157"/>
+      <c r="D6" s="157"/>
+      <c r="E6" s="158"/>
+      <c r="F6" s="127" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" s="128"/>
+      <c r="H6" s="128"/>
+      <c r="I6" s="128"/>
+      <c r="J6" s="41"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="32" t="s">
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="46"/>
-      <c r="H7" s="46"/>
-      <c r="I7" s="46"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
       <c r="J7" s="11"/>
     </row>
-    <row r="8" spans="1:10" ht="14.25">
-      <c r="A8" s="47" t="s">
+    <row r="8" spans="1:10">
+      <c r="A8" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="49"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="49"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
       <c r="J8" s="11"/>
     </row>
-    <row r="9" spans="1:10" ht="14.25">
-      <c r="A9" s="154" t="s">
+    <row r="9" spans="1:10">
+      <c r="A9" s="162" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="155"/>
-      <c r="C9" s="155"/>
-      <c r="D9" s="155"/>
-      <c r="E9" s="156"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="49"/>
+      <c r="B9" s="163"/>
+      <c r="C9" s="163"/>
+      <c r="D9" s="163"/>
+      <c r="E9" s="164"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="46"/>
       <c r="J9" s="11"/>
     </row>
-    <row r="10" spans="1:10" ht="14.25">
-      <c r="A10" s="154"/>
-      <c r="B10" s="155"/>
-      <c r="C10" s="155"/>
-      <c r="D10" s="155"/>
-      <c r="E10" s="156"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="49"/>
+    <row r="10" spans="1:10">
+      <c r="A10" s="162"/>
+      <c r="B10" s="163"/>
+      <c r="C10" s="163"/>
+      <c r="D10" s="163"/>
+      <c r="E10" s="164"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="46"/>
       <c r="J10" s="11"/>
     </row>
-    <row r="11" spans="1:10" ht="14.25">
+    <row r="11" spans="1:10">
       <c r="A11" s="1"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="46"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="34"/>
       <c r="J11" s="11"/>
     </row>
-    <row r="12" spans="1:10" ht="16.5">
-      <c r="A12" s="44" t="s">
+    <row r="12" spans="1:10">
+      <c r="A12" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="48"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="51"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="48"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="46"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
       <c r="J12" s="11"/>
     </row>
-    <row r="13" spans="1:10" ht="16.5">
-      <c r="A13" s="47" t="s">
+    <row r="13" spans="1:10">
+      <c r="A13" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="51"/>
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="48"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="46"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
       <c r="J13" s="11"/>
     </row>
-    <row r="14" spans="1:10" ht="14.25">
-      <c r="A14" s="47"/>
-      <c r="B14" s="52"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
+    <row r="14" spans="1:10">
+      <c r="A14" s="44"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
       <c r="J14" s="11"/>
     </row>
-    <row r="15" spans="1:10" ht="14.25">
-      <c r="A15" s="41"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="164"/>
-      <c r="G15" s="164"/>
+    <row r="15" spans="1:10">
+      <c r="A15" s="39"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="149"/>
+      <c r="G15" s="149"/>
       <c r="H15" s="4"/>
-      <c r="I15" s="54"/>
+      <c r="I15" s="50"/>
       <c r="J15" s="11"/>
     </row>
-    <row r="16" spans="1:10" ht="14.25">
-      <c r="A16" s="31" t="s">
+    <row r="16" spans="1:10">
+      <c r="A16" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="32" t="s">
+      <c r="B16" s="30"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="55"/>
-      <c r="F16" s="164"/>
-      <c r="G16" s="164"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="149"/>
+      <c r="G16" s="149"/>
       <c r="H16" s="5"/>
-      <c r="I16" s="46"/>
+      <c r="I16" s="34"/>
       <c r="J16" s="11"/>
     </row>
-    <row r="17" spans="1:10" ht="14.25">
-      <c r="A17" s="158"/>
-      <c r="B17" s="159"/>
-      <c r="C17" s="160"/>
-      <c r="D17" s="158"/>
-      <c r="E17" s="160"/>
-      <c r="F17" s="164"/>
-      <c r="G17" s="164"/>
+    <row r="17" spans="1:10">
+      <c r="A17" s="150"/>
+      <c r="B17" s="151"/>
+      <c r="C17" s="152"/>
+      <c r="D17" s="150"/>
+      <c r="E17" s="152"/>
+      <c r="F17" s="149"/>
+      <c r="G17" s="149"/>
       <c r="H17" s="5"/>
-      <c r="I17" s="46"/>
+      <c r="I17" s="34"/>
       <c r="J17" s="11"/>
     </row>
-    <row r="18" spans="1:10" ht="23.25">
-      <c r="A18" s="31" t="s">
+    <row r="18" spans="1:10" ht="31.2">
+      <c r="A18" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="56"/>
-      <c r="C18" s="57"/>
-      <c r="D18" s="117" t="s">
+      <c r="B18" s="45"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="109" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="58"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="46"/>
+      <c r="E18" s="53"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
       <c r="J18" s="11"/>
     </row>
-    <row r="19" spans="1:10" ht="14.25">
-      <c r="A19" s="158"/>
-      <c r="B19" s="159"/>
-      <c r="C19" s="160"/>
-      <c r="D19" s="149"/>
-      <c r="E19" s="150"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="42"/>
+    <row r="19" spans="1:10">
+      <c r="A19" s="150"/>
+      <c r="B19" s="151"/>
+      <c r="C19" s="152"/>
+      <c r="D19" s="140"/>
+      <c r="E19" s="141"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="40"/>
       <c r="J19" s="11"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="173" t="s">
+      <c r="A20" s="144" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="174" t="s">
+      <c r="B20" s="145" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="174" t="s">
+      <c r="C20" s="145" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="157" t="s">
+      <c r="D20" s="165" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="157"/>
-      <c r="F20" s="151" t="s">
+      <c r="E20" s="165"/>
+      <c r="F20" s="159" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="151" t="s">
+      <c r="G20" s="159" t="s">
         <v>18</v>
       </c>
-      <c r="H20" s="119" t="s">
+      <c r="H20" s="111" t="s">
         <v>59</v>
       </c>
-      <c r="I20" s="119" t="s">
+      <c r="I20" s="111" t="s">
         <v>58</v>
       </c>
-      <c r="J20" s="152" t="s">
+      <c r="J20" s="160" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:10">
-      <c r="A21" s="173"/>
-      <c r="B21" s="174"/>
-      <c r="C21" s="174"/>
-      <c r="D21" s="157"/>
-      <c r="E21" s="157"/>
-      <c r="F21" s="151"/>
-      <c r="G21" s="151"/>
-      <c r="H21" s="119" t="s">
+      <c r="A21" s="144"/>
+      <c r="B21" s="145"/>
+      <c r="C21" s="145"/>
+      <c r="D21" s="165"/>
+      <c r="E21" s="165"/>
+      <c r="F21" s="159"/>
+      <c r="G21" s="159"/>
+      <c r="H21" s="111" t="s">
         <v>37</v>
       </c>
-      <c r="I21" s="119" t="s">
+      <c r="I21" s="111" t="s">
         <v>37</v>
       </c>
-      <c r="J21" s="153"/>
-    </row>
-    <row r="22" spans="1:10" s="79" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A22" s="28">
+      <c r="J21" s="161"/>
+    </row>
+    <row r="22" spans="1:10" s="74" customFormat="1" ht="18.75" customHeight="1">
+      <c r="A22" s="27">
         <v>1</v>
       </c>
-      <c r="B22" s="75" t="str">
+      <c r="B22" s="70" t="str">
         <f>INVOICE!C20</f>
-        <v xml:space="preserve">2250303826/1.1 </v>
-      </c>
-      <c r="C22" s="75" t="str">
+        <v xml:space="preserve">2250303826.1.1 </v>
+      </c>
+      <c r="C22" s="70" t="str">
         <f>INVOICE!B20</f>
         <v xml:space="preserve">48310010VS   </v>
       </c>
-      <c r="D22" s="172" t="str">
+      <c r="D22" s="143" t="str">
         <f>INVOICE!D20</f>
         <v>蜂鸣器</v>
       </c>
-      <c r="E22" s="172"/>
-      <c r="F22" s="76">
+      <c r="E22" s="143"/>
+      <c r="F22" s="71">
         <f>INVOICE!E20</f>
         <v>5000</v>
       </c>
-      <c r="G22" s="77" t="s">
+      <c r="G22" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="H22" s="78">
+      <c r="H22" s="73">
         <v>2.5</v>
       </c>
-      <c r="I22" s="78">
+      <c r="I22" s="73">
         <v>5</v>
       </c>
-      <c r="J22" s="74" t="s">
+      <c r="J22" s="69" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="20.25" customHeight="1" thickBot="1">
       <c r="A23" s="7"/>
       <c r="B23" s="8"/>
-      <c r="C23" s="59"/>
-      <c r="D23" s="59"/>
-      <c r="E23" s="59"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="59"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="62"/>
-      <c r="J23" s="63"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="54"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="58"/>
     </row>
     <row r="24" spans="1:10">
-      <c r="A24" s="64">
+      <c r="A24" s="59">
         <f>SUM(A22:A23)</f>
         <v>1</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="56"/>
-      <c r="D24" s="171" t="s">
+      <c r="C24" s="45"/>
+      <c r="D24" s="142" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="171"/>
-      <c r="F24" s="129">
+      <c r="E24" s="142"/>
+      <c r="F24" s="10">
         <f>SUM(F22:F23)</f>
         <v>5000</v>
       </c>
       <c r="G24" s="10"/>
-      <c r="H24" s="65">
+      <c r="H24" s="60">
         <f>SUM(H22:H23)</f>
         <v>2.5</v>
       </c>
-      <c r="I24" s="65">
+      <c r="I24" s="60">
         <f>SUM(I22:I23)</f>
         <v>5</v>
       </c>
-      <c r="J24" s="66">
+      <c r="J24" s="61">
         <f>0.42*0.355*0.365*A24</f>
         <v>5.4421499999999991E-2</v>
       </c>
     </row>
     <row r="25" spans="1:10">
-      <c r="A25" s="67"/>
-      <c r="E25" s="68" t="s">
+      <c r="A25" s="62"/>
+      <c r="E25" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="F25" s="115">
+      <c r="F25" s="107">
         <f>A24</f>
         <v>1</v>
       </c>
-      <c r="J25" s="131"/>
+      <c r="J25" s="122"/>
     </row>
     <row r="26" spans="1:10" ht="24">
-      <c r="A26" s="67"/>
-      <c r="E26" s="116" t="s">
+      <c r="A26" s="62"/>
+      <c r="E26" s="108" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="118" t="s">
+      <c r="F26" s="110" t="s">
         <v>56</v>
       </c>
-      <c r="J26" s="69"/>
+      <c r="J26" s="64"/>
     </row>
     <row r="27" spans="1:10">
-      <c r="A27" s="67"/>
-      <c r="E27" s="68"/>
-      <c r="F27" s="70"/>
-      <c r="J27" s="69"/>
+      <c r="A27" s="62"/>
+      <c r="E27" s="63"/>
+      <c r="F27" s="65"/>
+      <c r="J27" s="64"/>
     </row>
     <row r="28" spans="1:10">
-      <c r="A28" s="71"/>
-      <c r="B28" s="72"/>
-      <c r="C28" s="72"/>
-      <c r="D28" s="72"/>
-      <c r="E28" s="72"/>
-      <c r="F28" s="72"/>
-      <c r="G28" s="72"/>
-      <c r="H28" s="72"/>
-      <c r="I28" s="72"/>
-      <c r="J28" s="73"/>
-    </row>
-    <row r="39" spans="5:5" ht="18.75">
-      <c r="E39" s="114" t="s">
+      <c r="A28" s="66"/>
+      <c r="B28" s="67"/>
+      <c r="C28" s="67"/>
+      <c r="D28" s="67"/>
+      <c r="E28" s="67"/>
+      <c r="F28" s="67"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="67"/>
+      <c r="I28" s="67"/>
+      <c r="J28" s="68"/>
+    </row>
+    <row r="39" spans="5:5" ht="19.8">
+      <c r="E39" s="106" t="s">
         <v>61</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="A9:E10"/>
+    <mergeCell ref="D20:E21"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:E19"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F16:G16"/>
@@ -2809,13 +2818,11 @@
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="A4:E6"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="A9:E10"/>
-    <mergeCell ref="D20:E21"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>